<commit_message>
Añadir gráfica MD2 con media de réplicas biológicas (MD2 1 y 2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQBVykGVcP6ajBzzUzdzHZ
</commit_message>
<xml_diff>
--- a/qPCR_analisis_MD2_MD3.xlsx
+++ b/qPCR_analisis_MD2_MD3.xlsx
@@ -182,6 +182,176 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>MD2 7 días: media de réplicas biológicas (MD2 1 y 2) vs 0d MD2, YWHAZ</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!J38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>Resumen!$L$39:$L$43</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>Resumen!$L$39:$L$43</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$I$39:$I$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$J$39:$J$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!K38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>Resumen!$M$39:$M$43</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>Resumen!$M$39:$M$43</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$I$39:$I$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$K$39:$K$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Gen</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <logBase val="10"/>
+          <orientation val="minMax"/>
+          <min val="0.1"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>RQ (2^-ΔΔCt)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -390,7 +560,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -601,6 +771,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -5270,7 +5462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5284,6 +5476,7 @@
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6530,6 +6723,157 @@
       <c r="K34" s="7">
         <f>SUMIFS($F$4:$F$28,$A$4:$A$28,K29,$B$4:$B$28,$I34)</f>
         <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="I37" s="14" t="inlineStr">
+        <is>
+          <t>MD2 7d – réplicas biológicas (MD2 1 y MD2 2): media y SD entre las dos</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Control 0d MD2</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>7d MD2 (media MD2 1 y 2)</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>SD control</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>SD entre réplicas (n=2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="J39" s="7">
+        <f>J5</f>
+        <v/>
+      </c>
+      <c r="K39" s="7">
+        <f>AVERAGE(K5,L5)</f>
+        <v/>
+      </c>
+      <c r="L39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="7">
+        <f>STDEV(K5,L5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="J40" s="7">
+        <f>J6</f>
+        <v/>
+      </c>
+      <c r="K40" s="7">
+        <f>AVERAGE(K6,L6)</f>
+        <v/>
+      </c>
+      <c r="L40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="7">
+        <f>STDEV(K6,L6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="J41" s="7">
+        <f>J7</f>
+        <v/>
+      </c>
+      <c r="K41" s="7">
+        <f>AVERAGE(K7,L7)</f>
+        <v/>
+      </c>
+      <c r="L41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="7">
+        <f>STDEV(K7,L7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="J42" s="7">
+        <f>J8</f>
+        <v/>
+      </c>
+      <c r="K42" s="7">
+        <f>AVERAGE(K8,L8)</f>
+        <v/>
+      </c>
+      <c r="L42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="7">
+        <f>STDEV(K8,L8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="J43" s="7">
+        <f>J9</f>
+        <v/>
+      </c>
+      <c r="K43" s="7">
+        <f>AVERAGE(K9,L9)</f>
+        <v/>
+      </c>
+      <c r="L43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="7">
+        <f>STDEV(K9,L9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>El control (RQ=1 por definición) va sin barra de error. SD entre réplicas con n=2.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadir gráfica comparativa MD2 (media) vs MD3
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQBVykGVcP6ajBzzUzdzHZ
</commit_message>
<xml_diff>
--- a/qPCR_analisis_MD2_MD3.xlsx
+++ b/qPCR_analisis_MD2_MD3.xlsx
@@ -363,6 +363,176 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>7 días: MD2 (media de 2 réplicas biológicas) vs MD3, relativo a su control 0d, YWHAZ</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!J49</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>Resumen!$L$50:$L$54</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>Resumen!$L$50:$L$54</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$I$50:$I$54</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$J$50:$J$54</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!K49</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>Resumen!$M$50:$M$54</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>Resumen!$M$50:$M$54</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$I$50:$I$54</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$K$50:$K$54</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Gen</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <logBase val="10"/>
+          <orientation val="minMax"/>
+          <min val="0.01"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>RQ (2^-ΔΔCt)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Expresión relativa MD2 (vs KerCT 0 días MD2), YWHAZ</a:t>
             </a:r>
           </a:p>
@@ -560,7 +730,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -793,6 +963,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -5462,7 +5654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6876,6 +7068,162 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="I48" s="14" t="inlineStr">
+        <is>
+          <t>MD2 (media de 1 y 2) vs MD3 a 7 días, cada uno relativo a su control 0d (RQ=1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>7d MD2 (media réplicas)</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>7d MD3</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>SD MD2 (entre réplicas, n=2)</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>SD MD3 (entre pocillos, n=1 biológica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="J50" s="7">
+        <f>K39</f>
+        <v/>
+      </c>
+      <c r="K50" s="7">
+        <f>K22</f>
+        <v/>
+      </c>
+      <c r="L50" s="7">
+        <f>M39</f>
+        <v/>
+      </c>
+      <c r="M50" s="7">
+        <f>K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="J51" s="7">
+        <f>K40</f>
+        <v/>
+      </c>
+      <c r="K51" s="7">
+        <f>K23</f>
+        <v/>
+      </c>
+      <c r="L51" s="7">
+        <f>M40</f>
+        <v/>
+      </c>
+      <c r="M51" s="7">
+        <f>K31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="J52" s="7">
+        <f>K41</f>
+        <v/>
+      </c>
+      <c r="K52" s="7">
+        <f>K24</f>
+        <v/>
+      </c>
+      <c r="L52" s="7">
+        <f>M41</f>
+        <v/>
+      </c>
+      <c r="M52" s="7">
+        <f>K32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="J53" s="7">
+        <f>K42</f>
+        <v/>
+      </c>
+      <c r="K53" s="7">
+        <f>K25</f>
+        <v/>
+      </c>
+      <c r="L53" s="7">
+        <f>M42</f>
+        <v/>
+      </c>
+      <c r="M53" s="7">
+        <f>K33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="J54" s="7">
+        <f>K43</f>
+        <v/>
+      </c>
+      <c r="K54" s="7">
+        <f>K26</f>
+        <v/>
+      </c>
+      <c r="L54" s="7">
+        <f>M43</f>
+        <v/>
+      </c>
+      <c r="M54" s="7">
+        <f>K34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>MD3 es una sola muestra: su barra de error refleja solo variación técnica entre pocillos, no biológica.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadir comparación MD2 vs Medio 3D (Prism) con gráficas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RQBVykGVcP6ajBzzUzdzHZ
</commit_message>
<xml_diff>
--- a/qPCR_analisis_MD2_MD3.xlsx
+++ b/qPCR_analisis_MD2_MD3.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Controles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Gráficas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Medio3D" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Comparación" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -87,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -105,6 +107,10 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -900,6 +906,385 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>7 días: MD2 vs Medio 3D (media ± SD entre réplicas biológicas)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Comparación'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>'Comparación'!$D$5:$D$9</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>'Comparación'!$D$5:$D$9</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Comparación'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comparación'!$B$5:$B$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Comparación'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>'Comparación'!$E$5:$E$9</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>'Comparación'!$E$5:$E$9</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Comparación'!$A$5:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comparación'!$C$5:$C$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Gen</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <logBase val="10"/>
+          <orientation val="minMax"/>
+          <min val="0.1"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>RQ (relativo a su día 0)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Medio 3D: evolución a 7, 14 y 20 días (media ± SD entre réplicas)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Comparación'!B12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>'Comparación'!$E$13:$E$18</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>'Comparación'!$E$13:$E$18</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Comparación'!$A$13:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comparación'!$B$13:$B$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Comparación'!C12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>'Comparación'!$F$13:$F$18</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>'Comparación'!$F$13:$F$18</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Comparación'!$A$13:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comparación'!$C$13:$C$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Comparación'!D12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <errBars>
+            <errBarType val="both"/>
+            <errValType val="cust"/>
+            <noEndCap val="0"/>
+            <minus>
+              <numRef>
+                <f>'Comparación'!$G$13:$G$18</f>
+              </numRef>
+            </minus>
+            <plus>
+              <numRef>
+                <f>'Comparación'!$G$13:$G$18</f>
+              </numRef>
+            </plus>
+          </errBars>
+          <cat>
+            <numRef>
+              <f>'Comparación'!$A$13:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Comparación'!$D$13:$D$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Gen</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <logBase val="10"/>
+          <orientation val="minMax"/>
+          <min val="0.01"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>RQ (relativo a su día 0)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -985,6 +1370,55 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -7249,4 +7683,1446 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Medio 3D (Prism, 2026-07-16): RQ relativo al día 0 de ese medio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Datos copiados del .prism (hojas "rep 1" y "rep2", azul = dato). Cada gen tiene 2 columnas por hoja. Supuesto: rep1 y rep2 son réplicas biológicas; dentro de cada una combino sus 2 columnas con media geométrica. Ojo: columna 1 es idéntica en rep1 y rep2, y las dos columnas difieren hasta 370 veces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>rep1 col 1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>rep1 col 2</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>rep2 col 1</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>rep2 col 2</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>rep1 (media geom.)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>rep2 (media geom.)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Media rep1-2</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>SD entre rep1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7">
+        <f>GEOMEAN(C5,D5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>GEOMEAN(E5,F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="7">
+        <f>AVERAGE(G5,H5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="7">
+        <f>STDEV(G5,H5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>518.4563801</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>1.38002677</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>518.4563801</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>63.3855219</v>
+      </c>
+      <c r="G6" s="7">
+        <f>GEOMEAN(C6,D6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="7">
+        <f>GEOMEAN(E6,F6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="7">
+        <f>AVERAGE(G6,H6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="7">
+        <f>STDEV(G6,H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>183.2161221</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>1639.91921</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>183.2161221</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>10186.2327</v>
+      </c>
+      <c r="G7" s="7">
+        <f>GEOMEAN(C7,D7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7">
+        <f>GEOMEAN(E7,F7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="7">
+        <f>AVERAGE(G7,H7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="7">
+        <f>STDEV(G7,H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>1.204569648</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>74.9980936</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>1.204569648</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>506.779904</v>
+      </c>
+      <c r="G8" s="7">
+        <f>GEOMEAN(C8,D8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="7">
+        <f>GEOMEAN(E8,F8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="7">
+        <f>AVERAGE(G8,H8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="7">
+        <f>STDEV(G8,H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="7">
+        <f>GEOMEAN(C9,D9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7">
+        <f>GEOMEAN(E9,F9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>AVERAGE(G9,H9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="7">
+        <f>STDEV(G9,H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1434.067349</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>3.56250986</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>1434.067349</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>214.892715</v>
+      </c>
+      <c r="G10" s="7">
+        <f>GEOMEAN(C10,D10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="7">
+        <f>GEOMEAN(E10,F10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="7">
+        <f>AVERAGE(G10,H10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="7">
+        <f>STDEV(G10,H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>2341.280147</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>273.190712</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>2341.280147</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>1972.33672</v>
+      </c>
+      <c r="G11" s="7">
+        <f>GEOMEAN(C11,D11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="7">
+        <f>GEOMEAN(E11,F11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>AVERAGE(G11,H11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="7">
+        <f>STDEV(G11,H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>5.693594117</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>18.2823582</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>5.693594117</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>118.225982</v>
+      </c>
+      <c r="G12" s="7">
+        <f>GEOMEAN(C12,D12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="7">
+        <f>GEOMEAN(E12,F12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="7">
+        <f>AVERAGE(G12,H12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="7">
+        <f>STDEV(G12,H12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="7">
+        <f>GEOMEAN(C13,D13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="7">
+        <f>GEOMEAN(E13,F13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="7">
+        <f>AVERAGE(G13,H13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="7">
+        <f>STDEV(G13,H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>2.04924663</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>4.98844718</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>2.04924663</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>4.98844718</v>
+      </c>
+      <c r="G14" s="7">
+        <f>GEOMEAN(C14,D14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="7">
+        <f>GEOMEAN(E14,F14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="7">
+        <f>AVERAGE(G14,H14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="7">
+        <f>STDEV(G14,H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>4.213340534</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>377.295873</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>4.213340534</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>377.295873</v>
+      </c>
+      <c r="G15" s="7">
+        <f>GEOMEAN(C15,D15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="7">
+        <f>GEOMEAN(E15,F15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="7">
+        <f>AVERAGE(G15,H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="7">
+        <f>STDEV(G15,H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>0.252368294</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>49.6153269</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>0.252368294</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>49.6153269</v>
+      </c>
+      <c r="G16" s="7">
+        <f>GEOMEAN(C16,D16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="7">
+        <f>GEOMEAN(E16,F16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="7">
+        <f>AVERAGE(G16,H16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="7">
+        <f>STDEV(G16,H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7">
+        <f>GEOMEAN(C17,D17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="7">
+        <f>GEOMEAN(E17,F17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="7">
+        <f>AVERAGE(G17,H17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="7">
+        <f>STDEV(G17,H17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>0.808314011</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>1.15453732</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <v>0.808314011</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>2.2412587</v>
+      </c>
+      <c r="G18" s="7">
+        <f>GEOMEAN(C18,D18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="7">
+        <f>GEOMEAN(E18,F18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="7">
+        <f>AVERAGE(G18,H18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="7">
+        <f>STDEV(G18,H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>47.51502437</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>4565.68891</v>
+      </c>
+      <c r="E19" s="16" t="n">
+        <v>47.51502437</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>14764.4908</v>
+      </c>
+      <c r="G19" s="7">
+        <f>GEOMEAN(C19,D19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7">
+        <f>GEOMEAN(E19,F19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="7">
+        <f>AVERAGE(G19,H19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>STDEV(G19,H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>5.096533244</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>198.573638</v>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>5.096533244</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>565.932597</v>
+      </c>
+      <c r="G20" s="7">
+        <f>GEOMEAN(C20,D20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="7">
+        <f>GEOMEAN(E20,F20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="7">
+        <f>AVERAGE(G20,H20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>STDEV(G20,H20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>KRT5</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="7">
+        <f>GEOMEAN(C21,D21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="7">
+        <f>GEOMEAN(E21,F21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="7">
+        <f>AVERAGE(G21,H21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="7">
+        <f>STDEV(G21,H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>KRT5</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>6.36581323</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>1.9515083</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <v>6.36581323</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>1.9515083</v>
+      </c>
+      <c r="G22" s="7">
+        <f>GEOMEAN(C22,D22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="7">
+        <f>GEOMEAN(E22,F22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="7">
+        <f>AVERAGE(G22,H22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="7">
+        <f>STDEV(G22,H22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>KRT5</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C23" s="16" t="n">
+        <v>0.178711827</v>
+      </c>
+      <c r="D23" s="16" t="n">
+        <v>0.15521415</v>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>0.178711827</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>0.15521415</v>
+      </c>
+      <c r="G23" s="7">
+        <f>GEOMEAN(C23,D23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="7">
+        <f>GEOMEAN(E23,F23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="7">
+        <f>AVERAGE(G23,H23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="7">
+        <f>STDEV(G23,H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>KRT5</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>0.22362597</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>0.5841091</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>0.22362597</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>0.5841091</v>
+      </c>
+      <c r="G24" s="7">
+        <f>GEOMEAN(C24,D24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="7">
+        <f>GEOMEAN(E24,F24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="7">
+        <f>AVERAGE(G24,H24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="7">
+        <f>STDEV(G24,H24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="7">
+        <f>GEOMEAN(C25,D25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="7">
+        <f>GEOMEAN(E25,F25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="7">
+        <f>AVERAGE(G25,H25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="7">
+        <f>STDEV(G25,H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>2.785870343</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>2.40481999</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>2.785870343</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>2.40481999</v>
+      </c>
+      <c r="G26" s="7">
+        <f>GEOMEAN(C26,D26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="7">
+        <f>GEOMEAN(E26,F26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="7">
+        <f>AVERAGE(G26,H26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="7">
+        <f>STDEV(G26,H26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>0.972730202</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>0.33321561</v>
+      </c>
+      <c r="E27" s="16" t="n">
+        <v>0.972730202</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>0.33321561</v>
+      </c>
+      <c r="G27" s="7">
+        <f>GEOMEAN(C27,D27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="7">
+        <f>GEOMEAN(E27,F27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="7">
+        <f>AVERAGE(G27,H27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="7">
+        <f>STDEV(G27,H27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>1.261520033</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <v>0.82330068</v>
+      </c>
+      <c r="E28" s="16" t="n">
+        <v>1.261520033</v>
+      </c>
+      <c r="F28" s="16" t="n">
+        <v>0.82330068</v>
+      </c>
+      <c r="G28" s="7">
+        <f>GEOMEAN(C28,D28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="7">
+        <f>GEOMEAN(E28,F28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="7">
+        <f>AVERAGE(G28,H28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="7">
+        <f>STDEV(G28,H28)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MD2 (7 días, media de MD2 1 y 2) vs Medio 3D (media de rep1 y rep2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cada medio va relativo a su propio día 0. SD = entre las 2 réplicas biológicas (n=2). KRT5 no se midió en MD2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>MD2 7d</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Medio 3D 7d</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>SD MD2</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>SD Medio 3D</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Medio 3D / MD2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B5" s="7">
+        <f>Resumen!K39</f>
+        <v/>
+      </c>
+      <c r="C5" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A5,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="D5" s="7">
+        <f>Resumen!M39</f>
+        <v/>
+      </c>
+      <c r="E5" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A5,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F5" s="7">
+        <f>IF(B5=0,"",C5/B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B6" s="7">
+        <f>Resumen!K40</f>
+        <v/>
+      </c>
+      <c r="C6" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A6,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>Resumen!M40</f>
+        <v/>
+      </c>
+      <c r="E6" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A6,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F6" s="7">
+        <f>IF(B6=0,"",C6/B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B7" s="7">
+        <f>Resumen!K41</f>
+        <v/>
+      </c>
+      <c r="C7" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A7,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>Resumen!M41</f>
+        <v/>
+      </c>
+      <c r="E7" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A7,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="7">
+        <f>IF(B7=0,"",C7/B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B8" s="7">
+        <f>Resumen!K42</f>
+        <v/>
+      </c>
+      <c r="C8" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A8,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>Resumen!M42</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A8,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="7">
+        <f>IF(B8=0,"",C8/B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B9" s="7">
+        <f>Resumen!K43</f>
+        <v/>
+      </c>
+      <c r="C9" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A9,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>Resumen!M43</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A9,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F9" s="7">
+        <f>IF(B9=0,"",C9/B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Evolución en el Medio 3D (media de rep1 y rep2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Gen</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>7 d</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>14 d</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>20 d</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>SD 7 d</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SD 14 d</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>SD 20 d</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>KRT1</t>
+        </is>
+      </c>
+      <c r="B13" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D13" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E13" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F13" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G13" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A13,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>KRT10</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E14" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F14" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A14,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>KRT2</t>
+        </is>
+      </c>
+      <c r="B15" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C15" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E15" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F15" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A15,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>IVL</t>
+        </is>
+      </c>
+      <c r="B16" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C16" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D16" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E16" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F16" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A16,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>KRT5</t>
+        </is>
+      </c>
+      <c r="B17" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C17" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D17" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E17" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F17" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G17" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A17,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>KRT14</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="C18" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="D18" s="7">
+        <f>SUMIFS(Medio3D!$I$5:$I$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+      <c r="E18" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,7)</f>
+        <v/>
+      </c>
+      <c r="F18" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,14)</f>
+        <v/>
+      </c>
+      <c r="G18" s="7">
+        <f>SUMIFS(Medio3D!$J$5:$J$28,Medio3D!$A$5:$A$28,$A18,Medio3D!$B$5:$B$28,20)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>